<commit_message>
Added Perimeter and Tariff to import abonents template
</commit_message>
<xml_diff>
--- a/assets/abonent-import-template_ar.xlsx
+++ b/assets/abonent-import-template_ar.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>ФИО</t>
   </si>
@@ -57,29 +57,35 @@
   <si>
     <t>Email</t>
   </si>
+  <si>
+    <t>Периметр</t>
+  </si>
+  <si>
+    <t>Тариф</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3">
     <font>
+      <sz val="11.000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="11.000000"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="24.000000"/>
+      <color indexed="2"/>
       <name val="Calibri"/>
-      <b/>
-      <color indexed="2"/>
-      <sz val="24.000000"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10.000000"/>
+      <color theme="1"/>
       <name val="Arial"/>
-      <color theme="1"/>
-      <sz val="10.000000"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1516,7 +1522,7 @@
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="4294967295" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1537,6 +1543,7 @@
     <col customWidth="1" min="10" max="10" width="16.42578125"/>
     <col customWidth="1" min="11" max="11" width="13.85546875"/>
     <col customWidth="1" min="12" max="12" width="12.28515625"/>
+    <col customWidth="1" min="15" max="15" width="12.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.199999999999999">
@@ -1582,8 +1589,12 @@
       <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
+      <c r="O1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
@@ -1628,7 +1639,7 @@
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="4294967295" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Floor to import abonents template
</commit_message>
<xml_diff>
--- a/assets/abonent-import-template_ar.xlsx
+++ b/assets/abonent-import-template_ar.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>ФИО</t>
   </si>
@@ -23,6 +23,9 @@
   </si>
   <si>
     <t>Адрес</t>
+  </si>
+  <si>
+    <t>Этаж</t>
   </si>
   <si>
     <t>Помещение</t>
@@ -1535,15 +1538,16 @@
     <col customWidth="1" min="1" max="1" width="27.7109375"/>
     <col customWidth="1" min="2" max="2" width="25.42578125"/>
     <col customWidth="1" min="3" max="3" width="25.85546875"/>
-    <col customWidth="1" min="4" max="4" width="16.7109375"/>
-    <col customWidth="1" min="5" max="5" width="23"/>
-    <col customWidth="1" min="6" max="6" width="18.42578125"/>
-    <col customWidth="1" min="7" max="8" width="22.42578125"/>
-    <col customWidth="1" min="9" max="9" width="20.7109375"/>
-    <col customWidth="1" min="10" max="10" width="16.42578125"/>
-    <col customWidth="1" min="11" max="11" width="13.85546875"/>
-    <col customWidth="1" min="12" max="12" width="12.28515625"/>
-    <col customWidth="1" min="15" max="15" width="12.140625"/>
+    <col customWidth="1" min="4" max="4" width="13.00390625"/>
+    <col customWidth="1" min="5" max="5" width="16.7109375"/>
+    <col customWidth="1" min="6" max="6" width="23"/>
+    <col customWidth="1" min="7" max="7" width="18.42578125"/>
+    <col customWidth="1" min="8" max="9" width="22.42578125"/>
+    <col customWidth="1" min="10" max="10" width="20.7109375"/>
+    <col customWidth="1" min="11" max="11" width="16.42578125"/>
+    <col customWidth="1" min="12" max="12" width="13.85546875"/>
+    <col customWidth="1" min="13" max="13" width="12.28515625"/>
+    <col customWidth="1" min="16" max="16" width="12.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.199999999999999">
@@ -1595,7 +1599,9 @@
       <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5"/>
+      <c r="Q1" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
       <c r="T1" s="5"/>
@@ -1606,6 +1612,7 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
       <c r="AA1" s="5"/>
+      <c r="AB1" s="5"/>
     </row>
     <row r="2" ht="15.75">
       <c r="A2" s="6"/>
@@ -1615,9 +1622,9 @@
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
-      <c r="H2" s="7"/>
+      <c r="H2" s="6"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="6"/>
+      <c r="J2" s="7"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
@@ -1635,6 +1642,7 @@
       <c r="Y2" s="6"/>
       <c r="Z2" s="6"/>
       <c r="AA2" s="6"/>
+      <c r="AB2" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>